<commit_message>
Ingestión de 4 documentos: mueve PDFs a Documentos/ y actualiza índice
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Datos/indice.xlsx
+++ b/Datos/indice.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BOB\Agente IA G9\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0760B61E-4E6B-47A3-ABAA-9BC7AF3E0584}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDD19F5-F04E-4C4E-A34F-77EE65F900FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{988E960D-89FA-4CB1-8671-18C4A779E4FE}"/>
+    <workbookView xWindow="360" yWindow="360" windowWidth="23010" windowHeight="12210" xr2:uid="{988E960D-89FA-4CB1-8671-18C4A779E4FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -98,9 +98,6 @@
     <t>Nombre Archivo</t>
   </si>
   <si>
-    <t>083 [TCS Rediris] Servicio de obtención de certificados de duración media (un año) [Wiki del STIC].pdf</t>
-  </si>
-  <si>
     <t>Instrucción de vacaciones y permisos PTGAS 2024.pdf</t>
   </si>
   <si>
@@ -122,9 +119,6 @@
     <t>2026-01</t>
   </si>
   <si>
-    <t>082 [Contrato Menor] Proceso de Contratación Menor [Wiki del STIC].pdf</t>
-  </si>
-  <si>
     <t>2026-02</t>
   </si>
   <si>
@@ -135,6 +129,12 @@
   </si>
   <si>
     <t>008 [GLPI] Gestión de tickets, proyectos y tareas [Wiki del STIC].pdf</t>
+  </si>
+  <si>
+    <t>082 [Contrato Menor] Proceso de Contratación Menor [Wiki del STIC].dokuwiki</t>
+  </si>
+  <si>
+    <t>083 [TCS Rediris] Servicio de obtención de certificados de duración media (un año) [Wiki del STIC].md</t>
   </si>
 </sst>
 </file>
@@ -543,8 +543,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.140625" customWidth="1"/>
-    <col min="2" max="2" width="50.42578125" customWidth="1"/>
-    <col min="3" max="3" width="71.140625" customWidth="1"/>
+    <col min="2" max="2" width="45.7109375" customWidth="1"/>
+    <col min="3" max="3" width="97.5703125" customWidth="1"/>
     <col min="4" max="4" width="56.7109375" customWidth="1"/>
     <col min="5" max="5" width="12.85546875" customWidth="1"/>
     <col min="7" max="7" width="12.42578125" customWidth="1"/>
@@ -575,13 +575,13 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
         <v>16</v>
       </c>
       <c r="C2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>15</v>
@@ -593,7 +593,7 @@
         <v>14</v>
       </c>
       <c r="G2" s="2">
-        <v>55153</v>
+        <v>46022</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
@@ -604,7 +604,7 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>17</v>
@@ -616,21 +616,21 @@
         <v>14</v>
       </c>
       <c r="G3" s="2">
-        <v>45651</v>
+        <v>45657</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B4" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" t="s">
         <v>24</v>
       </c>
-      <c r="C4" t="s">
-        <v>25</v>
-      </c>
       <c r="D4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="2">
         <v>46010</v>
@@ -644,13 +644,13 @@
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
         <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>9</v>
@@ -667,13 +667,13 @@
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>8</v>
@@ -690,13 +690,13 @@
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
         <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>7</v>

</xml_diff>

<commit_message>
Datos/indice.xlsx: actualiza el índice documental
Re-guardado del registro de documentos; las columnas Identificador y Estado
se mantienen sin cambios.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Datos/indice.xlsx
+++ b/Datos/indice.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\BOB\Agente IA G9\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EDD19F5-F04E-4C4E-A34F-77EE65F900FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46B76032-E74A-4258-8D0B-03A645ECDD28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="360" windowWidth="23010" windowHeight="12210" xr2:uid="{988E960D-89FA-4CB1-8671-18C4A779E4FE}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{988E960D-89FA-4CB1-8671-18C4A779E4FE}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>

</xml_diff>